<commit_message>
adding framework into repo
</commit_message>
<xml_diff>
--- a/ComcastCRMGUIFrameworkk/resource/testCase.xlsx
+++ b/ComcastCRMGUIFrameworkk/resource/testCase.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{EE95E531-9577-4E53-BC9D-904FEF7F32E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{3153F7D6-E2D5-41A4-A986-2931739870B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6C80BAAA-37DD-4FF9-A0B6-63EFABFF3705}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{6C80BAAA-37DD-4FF9-A0B6-63EFABFF3705}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -13,19 +13,10 @@
     <sheet name="contact" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:C20"/>
+  <oleSize ref="A1:K13"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>

</xml_diff>